<commit_message>
copy: polish delegated wording for PR #85
</commit_message>
<xml_diff>
--- a/docs/reviews/2026-10-22-t02-t03-tarot-copy-workbook.xlsx
+++ b/docs/reviews/2026-10-22-t02-t03-tarot-copy-workbook.xlsx
@@ -488,7 +488,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="49" customHeight="1">
+    <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Trạng thái</t>
@@ -496,7 +496,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>BẢN NHÁP chờ chủ sản phẩm duyệt. Chưa câu nào trong file này chạy trên app. Không có gì được nối vào engine hay vùng duyệt fallback cho tới khi owner duyệt; việc nối làm ở một PR riêng sau đó, giữ nguyên các bài đã rút (đóng băng theo phiên, US-20 AC15/AC17).</t>
+          <t xml:space="preserve">Đã có quyết định theo uỷ quyền ngày 26/10/2026; Codex chuốt câu chữ, Claude review bản sửa. Chưa nối vào app hay kho fallback. Việc nối làm ở PR riêng và giữ nguyên các bài đã rút.</t>
         </is>
       </c>
     </row>
@@ -6411,7 +6411,7 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="34" customHeight="1">
+    <row r="68" ht="48" customHeight="1">
       <c r="A68" s="5" t="inlineStr">
         <is>
           <t>T02-chia_se-self_care</t>
@@ -6491,7 +6491,7 @@
       </c>
       <c r="R68" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Cả tuần bạn trả lời mọi lời hỏi thăm bằng “mình ổn”, trong khi chuyện làm bạn bận lòng vẫn chưa kể với ai. (A ends in a dark room alone (heavy for a calm app); B is writing, not sharing). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Cả tuần bạn trả lời “mình ổn” mỗi khi được hỏi thăm, rồi chuyển sang chuyện khác. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -12554,7 +12554,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="34" customHeight="1">
+    <row r="6" ht="48" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>T03-nhan_loi-opening</t>
@@ -12628,7 +12628,7 @@
       </c>
       <c r="P6" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Mở lời: “Mình nhận nhé, mình chốt lại giờ giấc cụ thể với bạn được không?” (Both drafts are work-only (weekdays / hạn chót) but step renders for movie date, moving help, dinner). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Mở lời: “Mình nhận lời nhé, mình thống nhất thời gian cụ thể với bạn được không?” | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -17624,7 +17624,7 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="34" customHeight="1">
+    <row r="71" ht="48" customHeight="1">
       <c r="A71" s="5" t="inlineStr">
         <is>
           <t>T03-hen_gap-opening</t>
@@ -17698,7 +17698,7 @@
       </c>
       <c r="P71" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Mở lời: “Cuối tuần này bạn rảnh không, mình đi cà phê một chút nhé?” (A "Lâu rồi không gặp" wrong for new acquaintance row; B texting-only). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Mở lời: “Bạn rảnh lúc nào để mình hẹn gặp và nói chuyện một chút?” | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -20986,7 +20986,7 @@
         </is>
       </c>
     </row>
-    <row r="114" ht="34" customHeight="1">
+    <row r="114" ht="48" customHeight="1">
       <c r="A114" s="5" t="inlineStr">
         <is>
           <t>T03-gop_y-opening</t>
@@ -21060,7 +21060,7 @@
       </c>
       <c r="P114" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Mở lời: “Mình góp một ý nhỏ về chỗ này nhé, bạn thấy hợp thì dùng.” (A work-only (số liệu cũ), B partner-lateness only; step renders for all 4 topics). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Mở lời: “Bạn có muốn nghe một góp ý của mình về chuyện này không?” | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>

</xml_diff>